<commit_message>
Ya no es woke
</commit_message>
<xml_diff>
--- a/Albums List.xlsx
+++ b/Albums List.xlsx
@@ -2125,7 +2125,7 @@
     <t>Miracle Musical</t>
   </si>
   <si>
-    <t>Pop, Rap, Balad</t>
+    <t>Pop, Rap, Ballad</t>
   </si>
   <si>
     <t>When We Were Friends</t>
@@ -3556,7 +3556,7 @@
     <t>Laufey</t>
   </si>
   <si>
-    <t>Jazz Pop, Ballads, Modern Classical</t>
+    <t>Jazz Pop, Ballad, Modern Classical</t>
   </si>
   <si>
     <t>CASIOPEA</t>
@@ -17635,7 +17635,7 @@
       <c r="C307" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D307" s="15" t="s">
+      <c r="D307" s="13" t="s">
         <v>696</v>
       </c>
       <c r="E307" s="15" t="s">

</xml_diff>

<commit_message>
Fix GitHub Pages cache-busting and include updated Albums List.xlsx with .nojekyll
</commit_message>
<xml_diff>
--- a/Albums List.xlsx
+++ b/Albums List.xlsx
@@ -2935,7 +2935,7 @@
     <t>Ep.01-Causa</t>
   </si>
   <si>
-    <t>DELLAFUENTE, Taifa Yallah</t>
+    <t>DELLAFUENTE; Taifa Yallah</t>
   </si>
   <si>
     <t>Rock, Argentinean Rock, Hiphop/Rap</t>
@@ -22543,7 +22543,7 @@
       <c r="A421" s="15" t="s">
         <v>965</v>
       </c>
-      <c r="B421" s="15" t="s">
+      <c r="B421" s="13" t="s">
         <v>966</v>
       </c>
       <c r="C421" s="15" t="s">

</xml_diff>

<commit_message>
Split compound languages into individual languages matching genres behavior
</commit_message>
<xml_diff>
--- a/Albums List.xlsx
+++ b/Albums List.xlsx
@@ -13830,7 +13830,7 @@
         <v>2011.0</v>
       </c>
       <c r="G218" s="12" t="s">
-        <v>162</v>
+        <v>18</v>
       </c>
       <c r="H218" s="15"/>
       <c r="I218" s="17"/>
@@ -21397,8 +21397,8 @@
       <c r="F394" s="11">
         <v>2025.0</v>
       </c>
-      <c r="G394" s="16" t="s">
-        <v>116</v>
+      <c r="G394" s="12" t="s">
+        <v>22</v>
       </c>
       <c r="H394" s="15"/>
       <c r="I394" s="15"/>

</xml_diff>